<commit_message>
Add word "kombineres" to Random.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Random.xlsx
+++ b/12-06-2026-vokab/Random.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
-        <a:font script="Hang" typeface="맑은 고딕"/>
-        <a:font script="Hans" typeface="宋体"/>
-        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
+        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
+        <a:font script="Hans" typeface="å®ä½"/>
+        <a:font script="Hant" typeface="æ°ç´°æé«"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W1"/>
+  <dimension ref="A1:W2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -497,9 +497,80 @@
         <v>Lapses</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>7a31d1a6-074f-4495-bda3-5a26db386989</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-06-13</v>
+      </c>
+      <c r="C2" t="str">
+        <v>kombineres</v>
+      </c>
+      <c r="D2" t="str">
+        <v>kombinere</v>
+      </c>
+      <c r="E2" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F2" t="str">
+        <v/>
+      </c>
+      <c r="G2" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H2" t="str">
+        <v>[kʌmbiˈneˀʌ]</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://static.ordnet.dk/mp3/11027/11027007_2.mp3</v>
+      </c>
+      <c r="J2" t="str">
+        <v>sætte flere elementer sammen til en sammenhængende helhed</v>
+      </c>
+      <c r="K2" t="str">
+        <v>combine</v>
+      </c>
+      <c r="L2" t="str">
+        <v>*3-4-5 kamp kan ikke kombineres med Max’Rabat</v>
+      </c>
+      <c r="M2" t="str">
+        <v>Maximum Sønderborg | Book nemt sjove oplevelser online</v>
+      </c>
+      <c r="N2" t="str">
+        <v>https://bowlnfun.dk/centre/soenderborg/</v>
+      </c>
+      <c r="O2" t="str">
+        <v>https://bowlnfun.dk/centre/soenderborg/#:~:text=kombineres</v>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R2" t="str">
+        <v/>
+      </c>
+      <c r="S2" t="str">
+        <v/>
+      </c>
+      <c r="T2" t="str">
+        <v/>
+      </c>
+      <c r="U2" t="str">
+        <v/>
+      </c>
+      <c r="V2" t="str">
+        <v/>
+      </c>
+      <c r="W2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W2"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -508,23 +579,23 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q1"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -591,8 +662,8 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:B4"/>
   <cols>
-    <col min="1" max="1" width="16.83203125" customWidth="1"/>
-    <col min="2" max="2" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" customWidth="1" width="16.83203125"/>
+    <col min="2" max="2" customWidth="1" width="28.83203125"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Phone: add 1 entry in Random.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Random.xlsx
+++ b/12-06-2026-vokab/Random.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ï¼­ï¼³ ï¼°ã´ã·ãã¯"/>
-        <a:font script="Hang" typeface="ë§ì ê³ ë"/>
-        <a:font script="Hans" typeface="å®ä½"/>
-        <a:font script="Hant" typeface="æ°ç´°æé«"/>
+        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
+        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
+        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
+        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W2"/>
+  <dimension ref="A1:W3"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -418,7 +418,7 @@
     <col min="15" max="15" width="24.83203125" customWidth="1"/>
     <col min="16" max="16" width="18.83203125" customWidth="1"/>
     <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="18" max="18" width="14.83203125" customWidth="1"/>
     <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
     <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
     <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
@@ -568,9 +568,80 @@
         <v/>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>6e0580b6-f8cc-4e35-8214-d0a3a31400db</v>
+      </c>
+      <c r="B3" t="str">
+        <v>2026-06-13</v>
+      </c>
+      <c r="C3" t="str">
+        <v>pålæg</v>
+      </c>
+      <c r="D3" t="str">
+        <v/>
+      </c>
+      <c r="E3" t="str">
+        <v/>
+      </c>
+      <c r="F3" t="str">
+        <v/>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v/>
+      </c>
+      <c r="J3" t="str">
+        <v/>
+      </c>
+      <c r="K3" t="str">
+        <v/>
+      </c>
+      <c r="L3" t="str">
+        <v/>
+      </c>
+      <c r="M3" t="str">
+        <v/>
+      </c>
+      <c r="N3" t="str">
+        <v/>
+      </c>
+      <c r="O3" t="str">
+        <v/>
+      </c>
+      <c r="P3" t="str">
+        <v/>
+      </c>
+      <c r="Q3" t="str">
+        <v>pending</v>
+      </c>
+      <c r="R3" t="str">
+        <v/>
+      </c>
+      <c r="S3" t="str">
+        <v/>
+      </c>
+      <c r="T3" t="str">
+        <v/>
+      </c>
+      <c r="U3" t="str">
+        <v/>
+      </c>
+      <c r="V3" t="str">
+        <v/>
+      </c>
+      <c r="W3" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W3"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Phone: progress for 1 card in Random.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Random.xlsx
+++ b/12-06-2026-vokab/Random.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="Ã¯Â¼Â­Ã¯Â¼Â³ Ã¯Â¼Â°Ã£ÂÂ´Ã£ÂÂ·Ã£ÂÂÃ£ÂÂ¯"/>
-        <a:font script="Hang" typeface="Ã«Â§ÂÃ¬ÂÂ ÃªÂ³Â Ã«ÂÂ"/>
-        <a:font script="Hans" typeface="Ã¥Â®ÂÃ¤Â½Â"/>
-        <a:font script="Hant" typeface="Ã¦ÂÂ°Ã§Â´Â°Ã¦ÂÂÃ©Â«Â"/>
+        <a:font script="Jpan" typeface="ÃÂ¯ÃÂ¼ÃÂ­ÃÂ¯ÃÂ¼ÃÂ³ ÃÂ¯ÃÂ¼ÃÂ°ÃÂ£ÃÂÃÂ´ÃÂ£ÃÂÃÂ·ÃÂ£ÃÂÃÂÃÂ£ÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂ«ÃÂ§ÃÂÃÂ¬ÃÂÃÂ ÃÂªÃÂ³ÃÂ ÃÂ«ÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂ¥ÃÂ®ÃÂÃÂ¤ÃÂ½ÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂ¦ÃÂÃÂ°ÃÂ§ÃÂ´ÃÂ°ÃÂ¦ÃÂÃÂÃÂ©ÃÂ«ÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -401,29 +401,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:W3"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="14.83203125" customWidth="1"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="14.83203125"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -553,19 +553,19 @@
         <v/>
       </c>
       <c r="S2" t="str">
-        <v/>
+        <v>2026-06-13</v>
       </c>
       <c r="T2" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="U2" t="str">
-        <v/>
+        <v>2.3</v>
       </c>
       <c r="V2" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="W2" t="str">
-        <v/>
+        <v>0</v>
       </c>
     </row>
     <row r="3">

</xml_diff>

<commit_message>
Enrich 1 pending entry in Random.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Random.xlsx
+++ b/12-06-2026-vokab/Random.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ­ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ³ ÃÂÃÂ¯ÃÂÃÂ¼ÃÂÃÂ°ÃÂÃÂ£ÃÂÃÂÃÂÃÂ´ÃÂÃÂ£ÃÂÃÂÃÂÃÂ·ÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂ«ÃÂÃÂ§ÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂ ÃÂÃÂªÃÂÃÂ³ÃÂÃÂ ÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂ¥ÃÂÃÂ®ÃÂÃÂÃÂÃÂ¤ÃÂÃÂ½ÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂ¦ÃÂÃÂÃÂÃÂ°ÃÂÃÂ§ÃÂÃÂ´ÃÂÃÂ°ÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂ«ÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -579,28 +579,28 @@
         <v>pålæg</v>
       </c>
       <c r="D3" t="str">
-        <v/>
+        <v>pålæg</v>
       </c>
       <c r="E3" t="str">
-        <v/>
+        <v>substantiv</v>
       </c>
       <c r="F3" t="str">
-        <v/>
+        <v>et</v>
       </c>
       <c r="G3" t="str">
-        <v/>
+        <v>-get, -, -gene</v>
       </c>
       <c r="H3" t="str">
-        <v/>
+        <v>[ˈpʌˌlεˀg]</v>
       </c>
       <c r="I3" t="str">
-        <v/>
+        <v>https://static.ordnet.dk/mp3/11041/11041809_1.mp3</v>
       </c>
       <c r="J3" t="str">
-        <v/>
+        <v>madvarer som man lægger eller smører på udskåret brød, især skiver eller lag af pølse, postej, ost, tomat el.lign.</v>
       </c>
       <c r="K3" t="str">
-        <v/>
+        <v>toppings</v>
       </c>
       <c r="L3" t="str">
         <v/>
@@ -618,7 +618,7 @@
         <v/>
       </c>
       <c r="Q3" t="str">
-        <v>pending</v>
+        <v>ok</v>
       </c>
       <c r="R3" t="str">
         <v/>

</xml_diff>

<commit_message>
Phone: progress for 2 cards in Random.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Random.xlsx
+++ b/12-06-2026-vokab/Random.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -553,16 +553,16 @@
         <v/>
       </c>
       <c r="S2" t="str">
-        <v>2026-06-13</v>
+        <v>2026-06-16</v>
       </c>
       <c r="T2" t="str">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U2" t="str">
-        <v>2.1</v>
+        <v>2.25</v>
       </c>
       <c r="V2" t="str">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W2" t="str">
         <v>0</v>
@@ -624,19 +624,19 @@
         <v/>
       </c>
       <c r="S3" t="str">
-        <v/>
+        <v>2026-06-13</v>
       </c>
       <c r="T3" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="U3" t="str">
-        <v/>
+        <v>2.1</v>
       </c>
       <c r="V3" t="str">
-        <v/>
+        <v>0</v>
       </c>
       <c r="W3" t="str">
-        <v/>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add word "prikke" to Random.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Random.xlsx
+++ b/12-06-2026-vokab/Random.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,31 +399,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W3"/>
+  <dimension ref="A1:W4"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="14.83203125"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -639,9 +639,80 @@
         <v>0</v>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>2841d84f-1a49-40ff-bf28-dc4ffaea1933</v>
+      </c>
+      <c r="B4" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C4" t="str">
+        <v>prikke</v>
+      </c>
+      <c r="D4" t="str">
+        <v>prikke</v>
+      </c>
+      <c r="E4" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H4" t="str">
+        <v>[ˈpʁεgə]</v>
+      </c>
+      <c r="I4" t="str">
+        <v>https://static.ordnet.dk/mp3/11040/11040767_1.mp3</v>
+      </c>
+      <c r="J4" t="str">
+        <v>stikke let i eller gennem en overflade med en spids genstand</v>
+      </c>
+      <c r="K4" t="str">
+        <v>dot</v>
+      </c>
+      <c r="L4" t="str">
+        <v>I morgen kommer jeg til at gå rundt og prikke jer på skulderen for at få lovet at tage et billede af jer hver især.</v>
+      </c>
+      <c r="M4" t="str">
+        <v>(9) Facebook</v>
+      </c>
+      <c r="N4" t="str">
+        <v>https://www.facebook.com/</v>
+      </c>
+      <c r="O4" t="str">
+        <v>https://www.facebook.com/#:~:text=prikke</v>
+      </c>
+      <c r="P4" t="str">
+        <v/>
+      </c>
+      <c r="Q4" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R4" t="str">
+        <v/>
+      </c>
+      <c r="S4" t="str">
+        <v/>
+      </c>
+      <c r="T4" t="str">
+        <v/>
+      </c>
+      <c r="U4" t="str">
+        <v/>
+      </c>
+      <c r="V4" t="str">
+        <v/>
+      </c>
+      <c r="W4" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W4"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "lovet" to Random.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Random.xlsx
+++ b/12-06-2026-vokab/Random.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:W5"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -710,9 +710,80 @@
         <v/>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>db2b7be5-809b-4117-a167-a224e6ce4831</v>
+      </c>
+      <c r="B5" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C5" t="str">
+        <v>lovet</v>
+      </c>
+      <c r="D5" t="str">
+        <v>love</v>
+      </c>
+      <c r="E5" t="str">
+        <v>verbum</v>
+      </c>
+      <c r="F5" t="str">
+        <v/>
+      </c>
+      <c r="G5" t="str">
+        <v>-r, -de, -t</v>
+      </c>
+      <c r="H5" t="str">
+        <v>[ˈlɔːwə]</v>
+      </c>
+      <c r="I5" t="str">
+        <v>https://static.ordnet.dk/mp3/11030/11030997_1.mp3</v>
+      </c>
+      <c r="J5" t="str">
+        <v>give nogen et løfte</v>
+      </c>
+      <c r="K5" t="str">
+        <v>promised</v>
+      </c>
+      <c r="L5" t="str">
+        <v>I morgen kommer jeg til at gå rundt og prikke jer på skulderen for at få lovet at tage et billede af jer hver især.</v>
+      </c>
+      <c r="M5" t="str">
+        <v>(9) Facebook</v>
+      </c>
+      <c r="N5" t="str">
+        <v>https://www.facebook.com/</v>
+      </c>
+      <c r="O5" t="str">
+        <v>https://www.facebook.com/#:~:text=lovet</v>
+      </c>
+      <c r="P5" t="str">
+        <v/>
+      </c>
+      <c r="Q5" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R5" t="str">
+        <v/>
+      </c>
+      <c r="S5" t="str">
+        <v/>
+      </c>
+      <c r="T5" t="str">
+        <v/>
+      </c>
+      <c r="U5" t="str">
+        <v/>
+      </c>
+      <c r="V5" t="str">
+        <v/>
+      </c>
+      <c r="W5" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W5"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add phrase "hver især" to Random.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Random.xlsx
+++ b/12-06-2026-vokab/Random.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -401,29 +401,29 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:W5"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="18.83203125" customWidth="1"/>
-    <col min="4" max="4" width="14.83203125" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" customWidth="1"/>
-    <col min="6" max="6" width="8.83203125" customWidth="1"/>
-    <col min="7" max="7" width="26.83203125" customWidth="1"/>
-    <col min="8" max="8" width="16.83203125" customWidth="1"/>
-    <col min="9" max="9" width="18.83203125" customWidth="1"/>
-    <col min="10" max="10" width="36.83203125" customWidth="1"/>
-    <col min="11" max="11" width="36.83203125" customWidth="1"/>
-    <col min="12" max="12" width="50.83203125" customWidth="1"/>
-    <col min="13" max="13" width="24.83203125" customWidth="1"/>
-    <col min="14" max="14" width="24.83203125" customWidth="1"/>
-    <col min="15" max="15" width="24.83203125" customWidth="1"/>
-    <col min="16" max="16" width="18.83203125" customWidth="1"/>
-    <col min="17" max="17" width="10.83203125" customWidth="1"/>
-    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="18.83203125"/>
+    <col min="4" max="4" customWidth="1" width="14.83203125"/>
+    <col min="5" max="5" customWidth="1" width="11.83203125"/>
+    <col min="6" max="6" customWidth="1" width="8.83203125"/>
+    <col min="7" max="7" customWidth="1" width="26.83203125"/>
+    <col min="8" max="8" customWidth="1" width="16.83203125"/>
+    <col min="9" max="9" customWidth="1" width="18.83203125"/>
+    <col min="10" max="10" customWidth="1" width="36.83203125"/>
+    <col min="11" max="11" customWidth="1" width="36.83203125"/>
+    <col min="12" max="12" customWidth="1" width="50.83203125"/>
+    <col min="13" max="13" customWidth="1" width="24.83203125"/>
+    <col min="14" max="14" customWidth="1" width="24.83203125"/>
+    <col min="15" max="15" customWidth="1" width="24.83203125"/>
+    <col min="16" max="16" customWidth="1" width="18.83203125"/>
+    <col min="17" max="17" customWidth="1" width="10.83203125"/>
+    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -790,25 +790,25 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q1"/>
+  <dimension ref="A1:Q2"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="30.83203125"/>
-    <col min="4" max="4" customWidth="1" width="36.83203125"/>
-    <col min="5" max="5" customWidth="1" width="36.83203125"/>
-    <col min="6" max="6" customWidth="1" width="50.83203125"/>
-    <col min="7" max="7" customWidth="1" width="24.83203125"/>
-    <col min="8" max="8" customWidth="1" width="24.83203125"/>
-    <col min="9" max="9" customWidth="1" width="24.83203125"/>
-    <col min="10" max="10" customWidth="1" width="18.83203125"/>
-    <col min="11" max="11" customWidth="1" width="10.83203125"/>
-    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="30.83203125" customWidth="1"/>
+    <col min="4" max="4" width="36.83203125" customWidth="1"/>
+    <col min="5" max="5" width="36.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
+    <col min="7" max="7" width="24.83203125" customWidth="1"/>
+    <col min="8" max="8" width="24.83203125" customWidth="1"/>
+    <col min="9" max="9" width="24.83203125" customWidth="1"/>
+    <col min="10" max="10" width="18.83203125" customWidth="1"/>
+    <col min="11" max="11" width="10.83203125" customWidth="1"/>
+    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -864,9 +864,62 @@
         <v>Lapses</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>99c5a32b-c590-4ff0-b262-93133310c45b</v>
+      </c>
+      <c r="B2" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C2" t="str">
+        <v>hver især</v>
+      </c>
+      <c r="D2" t="str">
+        <v>hver=every · især=especially</v>
+      </c>
+      <c r="E2" t="str">
+        <v>each</v>
+      </c>
+      <c r="F2" t="str">
+        <v>I morgen kommer jeg til at gå rundt og prikke jer på skulderen for at få lovet at tage et billede af jer hver især.</v>
+      </c>
+      <c r="G2" t="str">
+        <v>(9) Facebook</v>
+      </c>
+      <c r="H2" t="str">
+        <v>https://www.facebook.com/</v>
+      </c>
+      <c r="I2" t="str">
+        <v>https://www.facebook.com/#:~:text=hver%20is%C3%A6r</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
+      <c r="K2" t="str">
+        <v>ok</v>
+      </c>
+      <c r="L2" t="str">
+        <v/>
+      </c>
+      <c r="M2" t="str">
+        <v/>
+      </c>
+      <c r="N2" t="str">
+        <v/>
+      </c>
+      <c r="O2" t="str">
+        <v/>
+      </c>
+      <c r="P2" t="str">
+        <v/>
+      </c>
+      <c r="Q2" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q2"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "kavalkade" to Random.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Random.xlsx
+++ b/12-06-2026-vokab/Random.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,31 +399,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W5"/>
+  <dimension ref="A1:W6"/>
   <cols>
-    <col min="1" max="1" customWidth="1" width="10.83203125"/>
-    <col min="2" max="2" customWidth="1" width="11.83203125"/>
-    <col min="3" max="3" customWidth="1" width="18.83203125"/>
-    <col min="4" max="4" customWidth="1" width="14.83203125"/>
-    <col min="5" max="5" customWidth="1" width="11.83203125"/>
-    <col min="6" max="6" customWidth="1" width="8.83203125"/>
-    <col min="7" max="7" customWidth="1" width="26.83203125"/>
-    <col min="8" max="8" customWidth="1" width="16.83203125"/>
-    <col min="9" max="9" customWidth="1" width="18.83203125"/>
-    <col min="10" max="10" customWidth="1" width="36.83203125"/>
-    <col min="11" max="11" customWidth="1" width="36.83203125"/>
-    <col min="12" max="12" customWidth="1" width="50.83203125"/>
-    <col min="13" max="13" customWidth="1" width="24.83203125"/>
-    <col min="14" max="14" customWidth="1" width="24.83203125"/>
-    <col min="15" max="15" customWidth="1" width="24.83203125"/>
-    <col min="16" max="16" customWidth="1" width="18.83203125"/>
-    <col min="17" max="17" customWidth="1" width="10.83203125"/>
-    <col min="18" max="18" customWidth="1" width="40.83203125" hidden="true"/>
-    <col min="19" max="19" customWidth="1" width="11.83203125" hidden="true"/>
-    <col min="20" max="20" customWidth="1" width="9.83203125" hidden="true"/>
-    <col min="21" max="21" customWidth="1" width="7.83203125" hidden="true"/>
-    <col min="22" max="22" customWidth="1" width="6.83203125" hidden="true"/>
-    <col min="23" max="23" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="1" max="1" width="10.83203125" customWidth="1"/>
+    <col min="2" max="2" width="11.83203125" customWidth="1"/>
+    <col min="3" max="3" width="18.83203125" customWidth="1"/>
+    <col min="4" max="4" width="14.83203125" customWidth="1"/>
+    <col min="5" max="5" width="11.83203125" customWidth="1"/>
+    <col min="6" max="6" width="8.83203125" customWidth="1"/>
+    <col min="7" max="7" width="26.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="18.83203125" customWidth="1"/>
+    <col min="10" max="10" width="36.83203125" customWidth="1"/>
+    <col min="11" max="11" width="36.83203125" customWidth="1"/>
+    <col min="12" max="12" width="50.83203125" customWidth="1"/>
+    <col min="13" max="13" width="24.83203125" customWidth="1"/>
+    <col min="14" max="14" width="24.83203125" customWidth="1"/>
+    <col min="15" max="15" width="24.83203125" customWidth="1"/>
+    <col min="16" max="16" width="18.83203125" customWidth="1"/>
+    <col min="17" max="17" width="10.83203125" customWidth="1"/>
+    <col min="18" max="18" width="40.83203125" customWidth="1" hidden="true"/>
+    <col min="19" max="19" width="11.83203125" customWidth="1" hidden="true"/>
+    <col min="20" max="20" width="9.83203125" customWidth="1" hidden="true"/>
+    <col min="21" max="21" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="22" max="22" width="6.83203125" customWidth="1" hidden="true"/>
+    <col min="23" max="23" width="7.83203125" customWidth="1" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -781,9 +781,80 @@
         <v/>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>c8843dbf-ede0-4e64-add6-905e167eceba</v>
+      </c>
+      <c r="B6" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C6" t="str">
+        <v>kavalkade</v>
+      </c>
+      <c r="D6" t="str">
+        <v>kavalkade</v>
+      </c>
+      <c r="E6" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F6" t="str">
+        <v>en</v>
+      </c>
+      <c r="G6" t="str">
+        <v>-n, -r, -rne</v>
+      </c>
+      <c r="H6" t="str">
+        <v>[kavalˈkæːðə]</v>
+      </c>
+      <c r="I6" t="str">
+        <v>https://static.ordnet.dk/mp3/11025/11025703_1.mp3</v>
+      </c>
+      <c r="J6" t="str">
+        <v>række af fx tv-udsendelser, opvisninger eller præsentationer om samme emne, med samme hovedperson, medvirkende el.lign.</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Cavalcade</v>
+      </c>
+      <c r="L6" t="str">
+        <v>Jeg har en idé om en lille kavalkade af opslag på Insta med billeder af os og et par stikord om hvem vi er. Det kan forhåbentlig give interesserede sjæle en idé om, hvor dejlig forskellig en flok vi er i koret. Det håber jeg, at I er med på.</v>
+      </c>
+      <c r="M6" t="str">
+        <v>(9) Facebook</v>
+      </c>
+      <c r="N6" t="str">
+        <v>https://www.facebook.com/</v>
+      </c>
+      <c r="O6" t="str">
+        <v>https://www.facebook.com/#:~:text=kavalkade</v>
+      </c>
+      <c r="P6" t="str">
+        <v/>
+      </c>
+      <c r="Q6" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R6" t="str">
+        <v/>
+      </c>
+      <c r="S6" t="str">
+        <v/>
+      </c>
+      <c r="T6" t="str">
+        <v/>
+      </c>
+      <c r="U6" t="str">
+        <v/>
+      </c>
+      <c r="V6" t="str">
+        <v/>
+      </c>
+      <c r="W6" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W6"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -792,23 +863,23 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:Q2"/>
   <cols>
-    <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="11.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="36.83203125" customWidth="1"/>
-    <col min="5" max="5" width="36.83203125" customWidth="1"/>
-    <col min="6" max="6" width="50.83203125" customWidth="1"/>
-    <col min="7" max="7" width="24.83203125" customWidth="1"/>
-    <col min="8" max="8" width="24.83203125" customWidth="1"/>
-    <col min="9" max="9" width="24.83203125" customWidth="1"/>
-    <col min="10" max="10" width="18.83203125" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" customWidth="1"/>
-    <col min="12" max="12" width="40.83203125" customWidth="1" hidden="true"/>
-    <col min="13" max="13" width="11.83203125" customWidth="1" hidden="true"/>
-    <col min="14" max="14" width="9.83203125" customWidth="1" hidden="true"/>
-    <col min="15" max="15" width="7.83203125" customWidth="1" hidden="true"/>
-    <col min="16" max="16" width="6.83203125" customWidth="1" hidden="true"/>
-    <col min="17" max="17" width="7.83203125" customWidth="1" hidden="true"/>
+    <col min="1" max="1" customWidth="1" width="10.83203125"/>
+    <col min="2" max="2" customWidth="1" width="11.83203125"/>
+    <col min="3" max="3" customWidth="1" width="30.83203125"/>
+    <col min="4" max="4" customWidth="1" width="36.83203125"/>
+    <col min="5" max="5" customWidth="1" width="36.83203125"/>
+    <col min="6" max="6" customWidth="1" width="50.83203125"/>
+    <col min="7" max="7" customWidth="1" width="24.83203125"/>
+    <col min="8" max="8" customWidth="1" width="24.83203125"/>
+    <col min="9" max="9" customWidth="1" width="24.83203125"/>
+    <col min="10" max="10" customWidth="1" width="18.83203125"/>
+    <col min="11" max="11" customWidth="1" width="10.83203125"/>
+    <col min="12" max="12" customWidth="1" width="40.83203125" hidden="true"/>
+    <col min="13" max="13" customWidth="1" width="11.83203125" hidden="true"/>
+    <col min="14" max="14" customWidth="1" width="9.83203125" hidden="true"/>
+    <col min="15" max="15" customWidth="1" width="7.83203125" hidden="true"/>
+    <col min="16" max="16" customWidth="1" width="6.83203125" hidden="true"/>
+    <col min="17" max="17" customWidth="1" width="7.83203125" hidden="true"/>
   </cols>
   <sheetData>
     <row r="1">

</xml_diff>

<commit_message>
Add word "opslag" to Random.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Random.xlsx
+++ b/12-06-2026-vokab/Random.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W6"/>
+  <dimension ref="A1:W7"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -852,9 +852,80 @@
         <v/>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>71a028c0-e913-411d-a88f-e934d3705da9</v>
+      </c>
+      <c r="B7" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C7" t="str">
+        <v>opslag</v>
+      </c>
+      <c r="D7" t="str">
+        <v>opslag</v>
+      </c>
+      <c r="E7" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F7" t="str">
+        <v>et</v>
+      </c>
+      <c r="G7" t="str">
+        <v>-et, -, -ene</v>
+      </c>
+      <c r="H7" t="str">
+        <v>[ˈʌbˌslæˀj]</v>
+      </c>
+      <c r="I7" t="str">
+        <v>https://static.ordnet.dk/mp3/11037/11037708_1.mp3</v>
+      </c>
+      <c r="J7" t="str">
+        <v>seddel, skilt el.lign. der hænges op på fx en opslagstavle eller en mur for at kunne læses af forbipasserende fx med en efterlysning eller en anden meddelelse</v>
+      </c>
+      <c r="K7" t="str">
+        <v>bulletin</v>
+      </c>
+      <c r="L7" t="str">
+        <v>Jeg har en idé om en lille kavalkade af opslag på Insta med billeder af os og et par stikord om hvem vi er. Det kan forhåbentlig give interesserede sjæle en idé om, hvor dejlig forskellig en flok vi er i koret. Det håber jeg, at I er med på.</v>
+      </c>
+      <c r="M7" t="str">
+        <v>(9) Facebook</v>
+      </c>
+      <c r="N7" t="str">
+        <v>https://www.facebook.com/</v>
+      </c>
+      <c r="O7" t="str">
+        <v>https://www.facebook.com/#:~:text=opslag</v>
+      </c>
+      <c r="P7" t="str">
+        <v/>
+      </c>
+      <c r="Q7" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R7" t="str">
+        <v/>
+      </c>
+      <c r="S7" t="str">
+        <v/>
+      </c>
+      <c r="T7" t="str">
+        <v/>
+      </c>
+      <c r="U7" t="str">
+        <v/>
+      </c>
+      <c r="V7" t="str">
+        <v/>
+      </c>
+      <c r="W7" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W7"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "stikord" to Random.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Random.xlsx
+++ b/12-06-2026-vokab/Random.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W7"/>
+  <dimension ref="A1:W8"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -923,9 +923,80 @@
         <v/>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>7c28f9a5-b85d-437c-8f53-51d93971f067</v>
+      </c>
+      <c r="B8" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C8" t="str">
+        <v>stikord</v>
+      </c>
+      <c r="D8" t="str">
+        <v>stikord</v>
+      </c>
+      <c r="E8" t="str">
+        <v>substantiv</v>
+      </c>
+      <c r="F8" t="str">
+        <v>et</v>
+      </c>
+      <c r="G8" t="str">
+        <v>-et, -, -ene</v>
+      </c>
+      <c r="H8" t="str">
+        <v>[ˈsdegˌoˀɐ̯]</v>
+      </c>
+      <c r="I8" t="str">
+        <v>https://static.ordnet.dk/mp3/11050/11050270_1.mp3</v>
+      </c>
+      <c r="J8" t="str">
+        <v>det eller de sidste ord i en replik betragtet som signal til næste skuespiller om at begynde sin replik eller gå ind på scenen</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Keywords</v>
+      </c>
+      <c r="L8" t="str">
+        <v>Jeg har en idé om en lille kavalkade af opslag på Insta med billeder af os og et par stikord om hvem vi er. Det kan forhåbentlig give interesserede sjæle en idé om, hvor dejlig forskellig en flok vi er i koret. Det håber jeg, at I er med på.</v>
+      </c>
+      <c r="M8" t="str">
+        <v>(9) Facebook</v>
+      </c>
+      <c r="N8" t="str">
+        <v>https://www.facebook.com/</v>
+      </c>
+      <c r="O8" t="str">
+        <v>https://www.facebook.com/#:~:text=stikord</v>
+      </c>
+      <c r="P8" t="str">
+        <v/>
+      </c>
+      <c r="Q8" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R8" t="str">
+        <v/>
+      </c>
+      <c r="S8" t="str">
+        <v/>
+      </c>
+      <c r="T8" t="str">
+        <v/>
+      </c>
+      <c r="U8" t="str">
+        <v/>
+      </c>
+      <c r="V8" t="str">
+        <v/>
+      </c>
+      <c r="W8" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W8"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "forhåbentlig" to Random.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Random.xlsx
+++ b/12-06-2026-vokab/Random.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Arial"/>
         <a:font script="Hebr" typeface="Arial"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -399,7 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W8"/>
+  <dimension ref="A1:W9"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
     <col min="2" max="2" width="11.83203125" customWidth="1"/>
@@ -994,9 +994,80 @@
         <v/>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>c749bbbc-028c-4d45-bfa6-3d61c6539c28</v>
+      </c>
+      <c r="B9" t="str">
+        <v>2026-06-15</v>
+      </c>
+      <c r="C9" t="str">
+        <v>forhåbentlig</v>
+      </c>
+      <c r="D9" t="str">
+        <v>forhåbentlig</v>
+      </c>
+      <c r="E9" t="str">
+        <v>adjektiv</v>
+      </c>
+      <c r="F9" t="str">
+        <v/>
+      </c>
+      <c r="G9" t="str">
+        <v>-t, -e</v>
+      </c>
+      <c r="H9" t="str">
+        <v>[fʌˈhɔˀbənli]</v>
+      </c>
+      <c r="I9" t="str">
+        <v>https://static.ordnet.dk/mp3/11014/11014619_1.mp3</v>
+      </c>
+      <c r="J9" t="str">
+        <v>som man håber på vil blive resultatet</v>
+      </c>
+      <c r="K9" t="str">
+        <v>hopefully</v>
+      </c>
+      <c r="L9" t="str">
+        <v>Jeg har en idé om en lille kavalkade af opslag på Insta med billeder af os og et par stikord om hvem vi er. Det kan forhåbentlig give interesserede sjæle en idé om, hvor dejlig forskellig en flok vi er i koret. Det håber jeg, at I er med på.</v>
+      </c>
+      <c r="M9" t="str">
+        <v>(9) Facebook</v>
+      </c>
+      <c r="N9" t="str">
+        <v>https://www.facebook.com/</v>
+      </c>
+      <c r="O9" t="str">
+        <v>https://www.facebook.com/#:~:text=forh%C3%A5bentlig</v>
+      </c>
+      <c r="P9" t="str">
+        <v/>
+      </c>
+      <c r="Q9" t="str">
+        <v>ok</v>
+      </c>
+      <c r="R9" t="str">
+        <v/>
+      </c>
+      <c r="S9" t="str">
+        <v/>
+      </c>
+      <c r="T9" t="str">
+        <v/>
+      </c>
+      <c r="U9" t="str">
+        <v/>
+      </c>
+      <c r="V9" t="str">
+        <v/>
+      </c>
+      <c r="W9" t="str">
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:W8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:W9"/>
   </ignoredErrors>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add word "sjæle" to Random.xlsx
</commit_message>
<xml_diff>
--- a/12-06-2026-vokab/Random.xlsx
+++ b/12-06-2026-vokab/Random.xlsx
@@ -123,10 +123,10 @@
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
-        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
-        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ·ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯"/>
+        <a:font script="Hang" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¬ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂªÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hans" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¥ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ®ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¤ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ½ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
+        <a:font script="Hant" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ§ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¦ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ©ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ«ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ"/>
         <a:font script="Arab" typeface="Times New Roman"/>
         <a:font script="Hebr" typeface="Times New Roman"/>
         <a:font script="Thai" typeface="Tahoma"/>
@@ -158,10 +158,10 @@
         <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
-        <a:font script="Jpan" typeface="ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ­ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ³ ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¯ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ¼ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ°ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ´ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ£ÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂÃÂ